<commit_message>
Fix Portuguese: accents, grammar, suítes (not apartamentos) across all 27 posts
</commit_message>
<xml_diff>
--- a/instagram-27-posts-zapier.xlsx
+++ b/instagram-27-posts-zapier.xlsx
@@ -590,14 +590,14 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Tem dias que a gente precisa lembrar que esse tipo de coisa existe a 2 horas de Sao Paulo.
-Campo aberto. Brasa acesa. Mesa posta. Por do sol que nao precisa de filtro.
-E isso que a gente faz aqui no Recanto das Seriemas, em Sao Pedro, SP.
-📍 2h de Sao Paulo
-🛏️ Pousada com 6 apartamentos
+          <t>Tem dias que a gente precisa lembrar que esse tipo de coisa existe a 2 horas de São Paulo.
+Campo aberto. Brasa acesa. Mesa posta. Pôr do sol que não precisa de filtro.
+É isso que a gente faz aqui no Recanto das Seriemas, em São Pedro, SP.
+📍 2h de São Paulo
+🛏️ Pousada com 6 suítes
 🔥 Parrilla de lenha
-🍷 Vinhedo, piquenique e degustacao de vinhos
-Reserve seu proximo fim de semana. Link na bio.</t>
+🍷 Vinhedo, piquenique e degustação de vinhos
+Reserve seu próximo fim de semana. Link na bio.</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -657,16 +657,16 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Nao tem atalho.
+          <t>Não tem atalho.
 A brasa esquenta devagar. A lenha estala no ritmo certo.
-A carne descansa. O sal trabalha. A fumaca sobe.
-Mas ninguem tem pressa aqui.
-Enquanto o fogo trabalha, voce descansa, toma um vinho e observa o horizonte abrir.
-A parrilla de lenha nao e so uma tecnica — e um ritmo. E esse ritmo e o do Recanto das Seriemas.
+A carne descansa. O sal trabalha. A fumaça sobe.
+Mas ninguém tem pressa aqui.
+Enquanto o fogo trabalha, você descansa, toma um vinho e observa o horizonte abrir.
+A parrilla de lenha não é só uma técnica — é um ritmo. E esse ritmo é o do Recanto das Seriemas.
 🔥 Parrilla de lenha real
 🌿 990 metros de altitude
-📍 Sao Pedro, SP
-Sabados e domingos. Reserve no link da bio.</t>
+📍 São Pedro, SP
+Sábados e domingos. Reserve no link da bio.</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -726,14 +726,14 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>5 motivos para passar o proximo fim de semana no Recanto das Seriemas 👉
-1. 🔥 Uma parrilla de lenha real — carne no ponto, fumaca, brasa viva.
-2. 🍷 Piquenique no vinhedo com degustacao de vinhos, queijo fresco artesanal e pao de fermentacao natural — tudo feito aqui.
-3. 🧀 Queijo fresco produzido na propriedade, pao caseiro assado toda manha, bolo que sai do forno antes de voce acordar.
-4. 🌄 990 metros de altitude na Serra do Itaqueri. Vista panoramica. Por do sol que nao precisa de filtro.
-5. 🛏️ 6 apartamentos com varanda, rede e silencio. A 15 minutos de Brotas e 2h de SP.
-Qual desses e o seu motivo?
-📍 Sao Pedro, SP · Reserve no link da bio</t>
+          <t>5 motivos para passar o próximo fim de semana no Recanto das Seriemas 👉
+1. 🔥 Uma parrilla de lenha real — carne no ponto, fumaça, brasa viva.
+2. 🍷 Piquenique no vinhedo com degustação de vinhos, queijo fresco artesanal e pão de fermentação natural — tudo feito aqui.
+3. 🧀 Queijo fresco produzido na propriedade, pão caseiro assado toda manhã, bolo que sai do forno antes de você acordar.
+4. 🌄 990 metros de altitude na Serra do Itaqueri. Vista panorâmica. Pôr do sol que não precisa de filtro.
+5. 🛏️ 6 suítes com varanda, rede e silêncio. A 15 minutos de Brotas e 2h de SP.
+Qual desses é o seu motivo?
+📍 São Pedro, SP · Reserve no link da bio</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -778,7 +778,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>O prato — urgencia</t>
+          <t>O prato — urgência</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -793,12 +793,12 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Isso nao e um prato.
-E o resultado de 4 horas de brasa, lenha e atencao.
-Picanha. Linguica artesanal. Legumes na chapa. Farofa. Vinagrete. Abobora assada.
+          <t>Isso não é um prato.
+É o resultado de 4 horas de brasa, lenha e atenção.
+Picanha. Linguiça artesanal. Legumes na chapa. Farofa. Vinagrete. Abóbora assada.
 Da parrilla de lenha direto pra mesa — sem atalho, sem desculpa.
-🔥 Sabado o fogo ja ta aceso. Ultimas vagas do fim de semana.
-📅 Reserve no link da bio · Sao Pedro, SP</t>
+🔥 Sábado o fogo já tá aceso. Últimas vagas do fim de semana.
+📅 Reserve no link da bio · São Pedro, SP</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -843,7 +843,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>O vinhedo — experiencias</t>
+          <t>O vinhedo — experiências</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -858,12 +858,12 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Poucos sabem que em Sao Pedro existe um vinhedo.
+          <t>Poucos sabem que em São Pedro existe um vinhedo.
 Menos ainda sabem que ele fica a 30 metros da nossa parrilla.
-O vinhedo do Recanto esta crescendo — as parreiras ainda sao jovens. Mas a experiencia ja esta pronta: piquenique entre as vinhas com queijo artesanal, pao de fermentacao natural e vinhos selecionados. Tudo com a vista do vale na frente.
-E quando a primeira safra sair, quem ja veio vai poder dizer que estava aqui desde o comeco.
-🍷 Piquenique e degustacao disponiveis ja
-📍 Sao Pedro, SP · 990m de altitude · Serra do Itaqueri</t>
+O vinhedo do Recanto está crescendo — as parreiras ainda são jovens. Mas a experiência já está pronta: piquenique entre as vinhas com queijo artesanal, pão de fermentação natural e vinhos selecionados. Tudo com a vista do vale na frente.
+E quando a primeira safra sair, quem já veio vai poder dizer que estava aqui desde o começo.
+🍷 Piquenique e degustação disponíveis já
+📍 São Pedro, SP · 990m de altitude · Serra do Itaqueri</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -923,12 +923,12 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Mesa grande. Prato cheio. Conversa que nao acaba.
-E isso que acontece quando a gente junta fogo, campo e as pessoas certas.
-Nao existe foto que capture o momento em que todo mundo para de falar e da a primeira garfada.
+          <t>Mesa grande. Prato cheio. Conversa que não acaba.
+É isso que acontece quando a gente junta fogo, campo e as pessoas certas.
+Não existe foto que capture o momento em que todo mundo para de falar e dá a primeira garfada.
 Mas a gente tenta. 📸
-Hoje e sabado no Recanto. O fogo ta aceso, a mesa ta posta e o horizonte nao vai a lugar nenhum.
-📍 Sao Pedro, SP · Reserve o proximo: link na bio</t>
+Hoje é sábado no Recanto. O fogo tá aceso, a mesa tá posta e o horizonte não vai a lugar nenhum.
+📍 São Pedro, SP · Reserve o próximo: link na bio</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -973,7 +973,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Reserve o proximo</t>
+          <t>Reserve o próximo</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -988,16 +988,16 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Chega para almocar.
-Pode ser que voce queira ficar para o domingo.
-Pode ser que voce ja esteja planejando a proxima vez antes de ir embora.
-Isso acontece quando o lugar, a comida e o silencio combinam com o ritmo certo.
-Brasa, vinho, queijo e campo. A serie completa.
-📍 Recanto das Seriemas · Sao Pedro, SP
-🛏️ 6 apartamentos com varanda e rede
+          <t>Chega para almoçar.
+Pode ser que você queira ficar para o domingo.
+Pode ser que você já esteja planejando a próxima vez antes de ir embora.
+Isso acontece quando o lugar, a comida e o silêncio combinam com o ritmo certo.
+Brasa, vinho, queijo e campo. A série completa.
+📍 Recanto das Seriemas · São Pedro, SP
+🛏️ 6 suítes com varanda e rede
 🔥 Parrilla de lenha aos fins de semana
-🍷 Piquenique e degustacao no vinhedo
-Reserve o proximo fim de semana. Link na bio.</t>
+🍷 Piquenique e degustação no vinhedo
+Reserve o próximo fim de semana. Link na bio.</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -1057,13 +1057,13 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>A rede esta la.
-Voce abre a porta e ela esta ali, esperando. Com o vale inteiro na frente.
-Nao tem pressa. Nao tem horario. Nao tem ninguem cobrando nada.
-So voce, a rede e o som do campo.
-Todas as suites do Recanto tem varanda privativa com rede. E todas tem essa vista.
-🛏️ 6 apartamentos · Varanda com rede
-📍 Sao Pedro, SP · 2h de Sao Paulo</t>
+          <t>A rede está lá.
+Você abre a porta e ela está ali, esperando. Com o vale inteiro na frente.
+Não tem pressa. Não tem horário. Não tem ninguém cobrando nada.
+Só você, a rede e o som do campo.
+Todas as suítes do Recanto têm varanda privativa com rede. E todas têm essa vista.
+🛏️ 6 suítes · Varanda com rede
+📍 São Pedro, SP · 2h de São Paulo</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1108,7 +1108,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>A arvore centenaria</t>
+          <t>A árvore centenária</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -1123,12 +1123,12 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Essa arvore ja viu muita coisa.
-Ja viu a terra virar cafe. Viu o cafe virar pasto. Viu o pasto virar vinhedo.
-E agora viu a gente montar uma mesa embaixo dela, servir parrilla de lenha e receber gente que vem de longe so pra sentar aqui.
-Algumas coisas levam tempo. Essa arvore sabe disso melhor que ninguem.
-🌳 Mesa ao ar livre sob a arvore centenaria
-📍 Recanto das Seriemas · Sao Pedro, SP</t>
+          <t>Essa árvore já viu muita coisa.
+Já viu a terra virar café. Viu o café virar pasto. Viu o pasto virar vinhedo.
+E agora viu a gente montar uma mesa embaixo dela, servir parrilla de lenha e receber gente que vem de longe só pra sentar aqui.
+Algumas coisas levam tempo. Essa árvore sabe disso melhor que ninguém.
+🌳 Mesa ao ar livre sob a árvore centenária
+📍 Recanto das Seriemas · São Pedro, SP</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1173,7 +1173,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>990m — cafe com nevoa</t>
+          <t>990m — café com névoa</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -1189,13 +1189,13 @@
       <c r="J11" s="2" t="inlineStr">
         <is>
           <t>990 metros de altitude.
-As 7h da manha, a nevoa ainda cobre o campo.
-E o cafe ja esta na mesa.
-Queijo fresco feito aqui. Pao caseiro assado de manha. Bolo ainda quente. Frutas do dia. E a nevoa do lado de fora que some quando o sol chega.
-Tem lugares que a gente descobre e nao consegue mais ficar sem voltar.
-O Recanto das Seriemas e um deles.
-☁️ Sao Pedro, SP · 990m de altitude · 2h de Sao Paulo
-🛏️ Reserve seu proximo fim de semana · Link na bio</t>
+Às 7h da manhã, a névoa ainda cobre o campo.
+E o café já está na mesa.
+Queijo fresco feito aqui. Pão caseiro assado de manhã. Bolo ainda quente. Frutas do dia. E a névoa do lado de fora que some quando o sol chega.
+Tem lugares que a gente descobre e não consegue mais ficar sem voltar.
+O Recanto das Seriemas é um deles.
+☁️ São Pedro, SP · 990m de altitude · 2h de São Paulo
+🛏️ Reserve seu próximo fim de semana · Link na bio</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1256,13 +1256,13 @@
       <c r="J12" s="2" t="inlineStr">
         <is>
           <t>Esse queijo foi feito aqui.
-Nao comprado. Nao encomendado. Feito. No Recanto das Seriemas. Artesanalmente. Todos os dias.
-E servido fresco no cafe da manha — com o pao caseiro que sai do forno de manha e a geleia artesanal que acompanha.
-Quando a gente diz "producao propria", e isso que a gente quer dizer.
+Não comprado. Não encomendado. Feito. No Recanto das Seriemas. Artesanalmente. Todos os dias.
+E servido fresco no café da manhã — com o pão caseiro que sai do forno de manhã e a geleia artesanal que acompanha.
+Quando a gente diz "produção própria", é isso que a gente quer dizer.
 🧀 Queijo fresco artesanal
-🍞 Pao caseiro diario
-☕ Cafe da manha incluso
-📍 Sao Pedro, SP · Reserve: link na bio</t>
+🍞 Pão caseiro diário
+☕ Café da manhã incluso
+📍 São Pedro, SP · Reserve: link na bio</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1307,7 +1307,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>O pao que sai do forno</t>
+          <t>O pão que sai do forno</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1322,15 +1322,15 @@
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>O pao e caseiro.
-Feito aqui, assado de manha, antes do cafe estar pronto.
-Com a crosta rustica que a gente gosta e o miolo que derrete com a manteiga.
-Do lado: geleia artesanal, requeijao e o queijo fresco que tambem e feito aqui no Recanto.
-As vezes o cafe da manha e o melhor momento do dia.
-🍞 Pao caseiro diario
+          <t>O pão é caseiro.
+Feito aqui, assado de manhã, antes do café estar pronto.
+Com a crosta rústica que a gente gosta e o miolo que derrete com a manteiga.
+Do lado: geleia artesanal, requeijão e o queijo fresco que também é feito aqui no Recanto.
+Às vezes o café da manhã é o melhor momento do dia.
+🍞 Pão caseiro diário
 🧀 Queijo fresco artesanal
-☕ Incluido em todas as diarias
-📍 Recanto das Seriemas · Sao Pedro, SP</t>
+☕ Incluído em todas as diárias
+📍 Recanto das Seriemas · São Pedro, SP</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Voce abre a porta e...</t>
+          <t>Você abre a porta e...</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -1390,11 +1390,11 @@
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Voce abre a porta e isso esta do outro lado.
-Nao e uma foto de banco de imagem. E a vista real do apartamento.
-O campo verde, o vale aberto e o silencio que so existe a 990 metros de altitude.
-Sao Pedro, SP. 2 horas de Sao Paulo. Um mundo inteiro de distancia.
-🏡 6 apartamentos com varanda · Todos com essa vista
+          <t>Você abre a porta e isso está do outro lado.
+Não é uma foto de banco de imagem. É a vista real da suíte.
+O campo verde, o vale aberto e o silêncio que só existe a 990 metros de altitude.
+São Pedro, SP. 2 horas de São Paulo. Um mundo inteiro de distância.
+🏡 6 suítes com varanda · Todas com essa vista
 📅 Reserve no link da bio</t>
         </is>
       </c>
@@ -1456,10 +1456,10 @@
       <c r="J15" s="2" t="inlineStr">
         <is>
           <t>O Recanto de noite.
-Sem pressa. Sem barulho. Sem ninguem pedindo nada.
-So o som do campo, as luzes baixas e a certeza de que amanha o cafe vai estar pronto quando voce acordar.
+Sem pressa. Sem barulho. Sem ninguém pedindo nada.
+Só o som do campo, as luzes baixas e a certeza de que amanhã o café vai estar pronto quando você acordar.
 Fica pro domingo.
-📍 Sao Pedro, SP · 990m · 2h de Sao Paulo
+📍 São Pedro, SP · 990m · 2h de São Paulo
 🛏️ Reserve: link na bio</t>
         </is>
       </c>
@@ -1505,7 +1505,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Embaixo da arvore</t>
+          <t>Embaixo da árvore</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1520,11 +1520,11 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Embaixo da arvore, com o vale na frente.
-A mesa posta. A parrilla servida. E o tipo de silencio que so existe quando voce esta longe o suficiente.
-Esse almoco nao e um evento. E o que acontece aqui todo fim de semana.
-📍 Recanto das Seriemas · Sao Pedro, SP
-🌳 Mesa ao ar livre sob a arvore centenaria</t>
+          <t>Embaixo da árvore, com o vale na frente.
+A mesa posta. A parrilla servida. É o tipo de silêncio que só existe quando você está longe o suficiente.
+Esse almoço não é um evento. É o que acontece aqui todo fim de semana.
+📍 Recanto das Seriemas · São Pedro, SP
+🌳 Mesa ao ar livre sob a árvore centenária</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -1585,9 +1585,9 @@
       <c r="J17" s="2" t="inlineStr">
         <is>
           <t>Depois do jantar, isso. Toda noite.
-O por do sol muda a cada dia. Mas a sensacao e sempre a mesma: voce para, respira e lembra por que veio.
-📍 Sao Pedro, SP · 990m de altitude
-🌅 O por do sol do Recanto das Seriemas</t>
+O pôr do sol muda a cada dia. Mas a sensação é sempre a mesma: você para, respira e lembra por que veio.
+📍 São Pedro, SP · 990m de altitude
+🌅 O pôr do sol do Recanto das Seriemas</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -1647,11 +1647,11 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>A varanda da sua suite 👉
-Nao importa qual apartamento voce escolher. Todos tem varanda privativa, rede e vista.
-A vista muda um pouco — vale direto, campo aberto, vinhedo de lado — mas o silencio e o mesmo.
-🛏️ 6 apartamentos · Varanda com rede em todos
-📍 Sao Pedro, SP · Reserve: link na bio</t>
+          <t>A varanda da sua suíte 👉
+Não importa qual suíte você escolher. Todas têm varanda privativa, rede e vista.
+A vista muda um pouco — vale direto, campo aberto, vinhedo de lado — mas o silêncio é o mesmo.
+🛏️ 6 suítes · Varanda com rede em todas
+📍 São Pedro, SP · Reserve: link na bio</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -1711,12 +1711,12 @@
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>Quando voce acordar, o bolo ja vai estar pronto.
-Feito de manha, ainda quente, com a banana da estacao caramelizando no forno enquanto voce dorme.
-E assim que comeca o dia no Recanto das Seriemas.
-Com bolo caseiro, queijo fresco da propria fazenda, pao feito aqui e o campo verde esperando do lado de fora.
-☀️ Todo fim de semana. Incluso na diaria.
-🏡 Pousada com 6 apartamentos · Sao Pedro, SP · 2h de Sao Paulo</t>
+          <t>Quando você acordar, o bolo já vai estar pronto.
+Feito de manhã, ainda quente, com a banana da estação caramelizando no forno enquanto você dorme.
+É assim que começa o dia no Recanto das Seriemas.
+Com bolo caseiro, queijo fresco da própria fazenda, pão feito aqui e o campo verde esperando do lado de fora.
+☀️ Todo fim de semana. Incluso na diária.
+🏡 Pousada com 6 suítes · São Pedro, SP · 2h de São Paulo</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -1776,12 +1776,12 @@
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>Plantamos o nosso vinhedo ha menos de dois anos.
-Ainda vai demorar para o primeiro vinho do Recanto estar pronto. E a gente nao tem pressa — vinho bom nao tem.
-Mas enquanto as vinhas crescem, a experiencia ja esta aqui: piquenique entre as parreiras com queijo fresco artesanal, pao de fermentacao natural e vinhos selecionados. Degustacao ao por do sol com vista para o vale.
-E quando a primeira safra sair, quem ja veio vai poder dizer que estava aqui desde o comeco.
-🍷 Piquenique e degustacao disponiveis
-📍 Recanto das Seriemas · Sao Pedro, SP</t>
+          <t>Plantamos o nosso vinhedo há menos de dois anos.
+Ainda vai demorar para o primeiro vinho do Recanto estar pronto. E a gente não tem pressa — vinho bom não tem.
+Mas enquanto as vinhas crescem, a experiência já está aqui: piquenique entre as parreiras com queijo fresco artesanal, pão de fermentação natural e vinhos selecionados. Degustação ao pôr do sol com vista para o vale.
+E quando a primeira safra sair, quem já veio vai poder dizer que estava aqui desde o começo.
+🍷 Piquenique e degustação disponíveis
+📍 Recanto das Seriemas · São Pedro, SP</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -1841,11 +1841,11 @@
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>Brasa, vinho, queijo e campo. A serie completa.
-📍 Recanto das Seriemas · Sao Pedro, SP
-🔥 Parrilla de lenha · Sabados e domingos
-🍷 Piquenique e degustacao no vinhedo
-🛏️ 6 apartamentos com varanda e rede
+          <t>Brasa, vinho, queijo e campo. A série completa.
+📍 Recanto das Seriemas · São Pedro, SP
+🔥 Parrilla de lenha · Sábados e domingos
+🍷 Piquenique e degustação no vinhedo
+🛏️ 6 suítes com varanda e rede
 Reserve: link na bio</t>
         </is>
       </c>
@@ -1891,7 +1891,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Vagas para o proximo FDS</t>
+          <t>Vagas para o próximo FDS</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -1906,12 +1906,12 @@
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>Restam vagas para o proximo fim de semana.
-🔥 Parrilla de lenha — sabado e domingo
-🍷 Piquenique e degustacao no vinhedo
-🧀 Cafe da manha com queijo fresco e pao artesanal
-🛏️ 6 apartamentos com varanda e rede
-📍 Sao Pedro, SP · 2h de Sao Paulo · 15 min de Brotas
+          <t>Restam vagas para o próximo fim de semana.
+🔥 Parrilla de lenha — sábado e domingo
+🍷 Piquenique e degustação no vinhedo
+🧀 Café da manhã com queijo fresco e pão artesanal
+🛏️ 6 suítes com varanda e rede
+📍 São Pedro, SP · 2h de São Paulo · 15 min de Brotas
 Reserve agora: link na bio. Quando lotar, lotou.</t>
         </is>
       </c>
@@ -1957,7 +1957,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Acordar aqui e assim</t>
+          <t>Acordar aqui é assim</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -1972,12 +1972,12 @@
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>Acordar aqui e assim.
-Ovos mexidos, queijo fresco feito no proprio Recanto, pao caseiro assado de manha, suco de laranja natural e o campo verde pela janela.
-Nao e "cafe da manha incluso na diaria".
-E a primeira refeicao do dia feita com o mesmo cuidado que a gente coloca na brasa do sabado.
+          <t>Acordar aqui é assim.
+Ovos mexidos, queijo fresco feito no próprio Recanto, pão caseiro assado de manhã, suco de laranja natural e o campo verde pela janela.
+Não é "café da manhã incluso na diária".
+É a primeira refeição do dia feita com o mesmo cuidado que a gente coloca na brasa do sábado.
 ☕ Todos os dias. Incluso.
-📍 Recanto das Seriemas · Sao Pedro, SP</t>
+📍 Recanto das Seriemas · São Pedro, SP</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
@@ -2022,7 +2022,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Carrossel cafe: 5 razoes</t>
+          <t>Carrossel café: 5 razões</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -2037,14 +2037,14 @@
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>5 razoes para nao pular o cafe da manha no Recanto 👉
-1. 🧀 O queijo fresco e feito aqui — producao propria, todo dia
-2. 🍞 O pao sai do forno de manha — voce sente o cheiro do quarto
-3. 🎂 O bolo e caseiro — banana, laranja, o que a estacao oferecer
+          <t>5 razões para não pular o café da manhã no Recanto 👉
+1. 🧀 O queijo fresco é feito aqui — produção própria, todo dia
+2. 🍞 O pão sai do forno de manhã — você sente o cheiro do quarto
+3. 🎂 O bolo é caseiro — banana, laranja, o que a estação oferecer
 4. ☕ Tudo incluso — sem surpresas, sem extras
-5. 🌄 A vista pela janela — campo verde, nevoa e o silencio da serra
-Tem cafe da manha. E tem o cafe da manha do Recanto.
-📍 Sao Pedro, SP · 990m de altitude
+5. 🌄 A vista pela janela — campo verde, névoa e o silêncio da serra
+Tem café da manhã. E tem o café da manhã do Recanto.
+📍 São Pedro, SP · 990m de altitude
 🛏️ Reserve: link na bio</t>
         </is>
       </c>
@@ -2105,11 +2105,11 @@
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>Queijo fresco artesanal. Pao de fermentacao natural. Geleia caseira. Uma garrafa de vinho. E o horizonte do interior de SP abrindo na sua frente.
-Isso e o Piquenique no Vinhedo do Recanto das Seriemas.
-As vinhas tem menos de dois anos — ainda estao crescendo. Mas a experiencia ja esta pronta — com tudo produzido aqui, na propriedade.
+          <t>Queijo fresco artesanal. Pão de fermentação natural. Geleia caseira. Uma garrafa de vinho. E o horizonte do interior de SP abrindo na sua frente.
+Isso é o Piquenique no Vinhedo do Recanto das Seriemas.
+As vinhas têm menos de dois anos — ainda estão crescendo. Mas a experiência já está pronta — com tudo produzido aqui, na propriedade.
 🍷 R$ 220 por casal · Sexta a domingo
-📍 Sao Pedro, SP · Reserve pelo WhatsApp: link na bio</t>
+📍 São Pedro, SP · Reserve pelo WhatsApp: link na bio</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
@@ -2154,7 +2154,7 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Estava no comeco</t>
+          <t>Estava no começo</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
@@ -2169,13 +2169,13 @@
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>Plantamos o nosso vinhedo ha menos de dois anos.
-Ainda vai demorar para o primeiro vinho do Recanto estar pronto. E a gente nao tem pressa — vinho bom nao tem.
-Mas enquanto as vinhas crescem, voce ja pode caminhar entre elas. Fazer um piquenique com vista para o vale. Degustar vinhos selecionados com o queijo e o pao que a gente produz aqui. Respirar o ar da Serra do Itaqueri.
-E colocar seu nome na lista dos que vao provar o primeiro vinho daqui.
-Algumas das melhores historias comecam antes do fim.
-📍 Recanto das Seriemas · Sao Pedro, SP
-🍷 Piquenique e degustacao disponiveis ja</t>
+          <t>Plantamos o nosso vinhedo há menos de dois anos.
+Ainda vai demorar para o primeiro vinho do Recanto estar pronto. E a gente não tem pressa — vinho bom não tem.
+Mas enquanto as vinhas crescem, você já pode caminhar entre elas. Fazer um piquenique com vista para o vale. Degustar vinhos selecionados com o queijo e o pão que a gente produz aqui. Respirar o ar da Serra do Itaqueri.
+E colocar seu nome na lista dos que vão provar o primeiro vinho daqui.
+Algumas das melhores histórias começam antes do fim.
+📍 Recanto das Seriemas · São Pedro, SP
+🍷 Piquenique e degustação disponíveis já</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
@@ -2235,11 +2235,11 @@
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>Enquanto a brasa trabalha, a gente aguarda do lado de ca.
-Cachaca da Vo Zepi. Um vinho bom. Um papo melhor ainda. E o som da lenha que crepita la atras.
-Isso e o intervalo perfeito entre a entrada e o prato principal no Recanto das Seriemas.
-🍾 Interior de SP · Sabados e domingos
-📍 Sao Pedro, SP · 2h de Sao Paulo</t>
+          <t>Enquanto a brasa trabalha, a gente aguarda do lado de cá.
+Cachaça da Vó Zepi. Um vinho bom. Um papo melhor ainda. E o som da lenha que crepita lá atrás.
+Isso é o intervalo perfeito entre a entrada e o prato principal no Recanto das Seriemas.
+🍾 Interior de SP · Sábados e domingos
+📍 São Pedro, SP · 2h de São Paulo</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
@@ -2299,12 +2299,12 @@
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>A vista da varanda hoje de manha.
-Campo verde, um rebanho la embaixo, e o silencio que Sao Paulo nao tem.
-Essa e a vista que espera do outro lado da janela no Recanto das Seriemas — 990 metros de altitude, interior paulista, 2 horas de casa.
-As vezes e preciso lembrar que isso existe.
-📍 Sao Pedro, SP
-🏠 Varanda privativa com rede em todos os apartamentos
+          <t>A vista da varanda hoje de manhã.
+Campo verde, um rebanho lá embaixo, e o silêncio que São Paulo não tem.
+Essa é a vista que espera do outro lado da janela no Recanto das Seriemas — 990 metros de altitude, interior paulista, 2 horas de casa.
+Às vezes é preciso lembrar que isso existe.
+📍 São Pedro, SP
+🏠 Varanda privativa com rede em todas as suítes
 📅 Reserve: link na bio</t>
         </is>
       </c>

</xml_diff>